<commit_message>
feat(users): allocate unique three-letter initials and shorten lab usernames
Directory and seed identities stay unique even after soft-delete, and lab
usernames match the short NIK-style ids used on the shared lab.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/deploy/apex-landing/seed-lab-module-users-200.xlsx
+++ b/deploy/apex-landing/seed-lab-module-users-200.xlsx
@@ -431,13 +431,11 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>username = ID 16 digit (identitas pusat)</t>
+          <t>username = ID login pendek (3101, 3102, …); external_user_id = ID 16 digit</t>
         </is>
       </c>
     </row>
@@ -448,9 +446,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -465,9 +461,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -478,7 +472,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ID range: 3100000000000001 … 3100000000000200</t>
+          <t>Login: 3101 … 31200 (identity 16 digit tetap di email/external_user_id)</t>
         </is>
       </c>
     </row>
@@ -556,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>3100000000000001</t>
+          <t>3101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -613,7 +607,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>3100000000000002</t>
+          <t>3102</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -670,7 +664,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>3100000000000003</t>
+          <t>3103</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -727,7 +721,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>3100000000000004</t>
+          <t>3104</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -784,7 +778,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3100000000000005</t>
+          <t>3105</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -841,7 +835,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>3100000000000006</t>
+          <t>3106</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -898,7 +892,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>3100000000000007</t>
+          <t>3107</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -955,7 +949,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>3100000000000008</t>
+          <t>3108</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1012,7 +1006,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>3100000000000009</t>
+          <t>3109</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1069,7 +1063,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>3100000000000010</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1126,7 +1120,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>3100000000000011</t>
+          <t>3111</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1183,7 +1177,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>3100000000000012</t>
+          <t>3112</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1240,7 +1234,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>3100000000000013</t>
+          <t>3113</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1297,7 +1291,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>3100000000000014</t>
+          <t>3114</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1354,7 +1348,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>3100000000000015</t>
+          <t>3115</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1411,7 +1405,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>3100000000000016</t>
+          <t>3116</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1468,7 +1462,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>3100000000000017</t>
+          <t>3117</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1525,7 +1519,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>3100000000000018</t>
+          <t>3118</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1582,7 +1576,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>3100000000000019</t>
+          <t>3119</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1639,7 +1633,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>3100000000000020</t>
+          <t>3120</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1696,7 +1690,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>3100000000000021</t>
+          <t>3121</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1753,7 +1747,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>3100000000000022</t>
+          <t>3122</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1810,7 +1804,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>3100000000000023</t>
+          <t>3123</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1867,7 +1861,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>3100000000000024</t>
+          <t>3124</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1924,7 +1918,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>3100000000000025</t>
+          <t>3125</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1981,7 +1975,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>3100000000000026</t>
+          <t>3126</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2038,7 +2032,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>3100000000000027</t>
+          <t>3127</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2095,7 +2089,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>3100000000000028</t>
+          <t>3128</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2152,7 +2146,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>3100000000000029</t>
+          <t>3129</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2209,7 +2203,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>3100000000000030</t>
+          <t>3130</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2266,7 +2260,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>3100000000000031</t>
+          <t>3131</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2323,7 +2317,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>3100000000000032</t>
+          <t>3132</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2380,7 +2374,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>3100000000000033</t>
+          <t>3133</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2437,7 +2431,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>3100000000000034</t>
+          <t>3134</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2494,7 +2488,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>3100000000000035</t>
+          <t>3135</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2551,7 +2545,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>3100000000000036</t>
+          <t>3136</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2608,7 +2602,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>3100000000000037</t>
+          <t>3137</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2665,7 +2659,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>3100000000000038</t>
+          <t>3138</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2722,7 +2716,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>3100000000000039</t>
+          <t>3139</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2779,7 +2773,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>3100000000000040</t>
+          <t>3140</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2836,7 +2830,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>3100000000000041</t>
+          <t>3141</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2893,7 +2887,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>3100000000000042</t>
+          <t>3142</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2950,7 +2944,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>3100000000000043</t>
+          <t>3143</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3007,7 +3001,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>3100000000000044</t>
+          <t>3144</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3064,7 +3058,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>3100000000000045</t>
+          <t>3145</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3121,7 +3115,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>3100000000000046</t>
+          <t>3146</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3178,7 +3172,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>3100000000000047</t>
+          <t>3147</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3235,7 +3229,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>3100000000000048</t>
+          <t>3148</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3292,7 +3286,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>3100000000000049</t>
+          <t>3149</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3349,7 +3343,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>3100000000000050</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3406,7 +3400,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>3100000000000051</t>
+          <t>3151</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3463,7 +3457,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>3100000000000052</t>
+          <t>3152</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3520,7 +3514,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>3100000000000053</t>
+          <t>3153</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3577,7 +3571,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>3100000000000054</t>
+          <t>3154</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3634,7 +3628,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>3100000000000055</t>
+          <t>3155</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3691,7 +3685,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>3100000000000056</t>
+          <t>3156</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3748,7 +3742,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>3100000000000057</t>
+          <t>3157</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3805,7 +3799,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>3100000000000058</t>
+          <t>3158</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3862,7 +3856,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>3100000000000059</t>
+          <t>3159</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3919,7 +3913,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>3100000000000060</t>
+          <t>3160</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3976,7 +3970,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>3100000000000061</t>
+          <t>3161</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4033,7 +4027,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>3100000000000062</t>
+          <t>3162</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -4090,7 +4084,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>3100000000000063</t>
+          <t>3163</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -4147,7 +4141,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>3100000000000064</t>
+          <t>3164</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4204,7 +4198,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>3100000000000065</t>
+          <t>3165</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -4261,7 +4255,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>3100000000000066</t>
+          <t>3166</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4318,7 +4312,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>3100000000000067</t>
+          <t>3167</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4375,7 +4369,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>3100000000000068</t>
+          <t>3168</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4432,7 +4426,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>3100000000000069</t>
+          <t>3169</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4489,7 +4483,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>3100000000000070</t>
+          <t>3170</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4546,7 +4540,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>3100000000000071</t>
+          <t>3171</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4603,7 +4597,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>3100000000000072</t>
+          <t>3172</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4660,7 +4654,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>3100000000000073</t>
+          <t>3173</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4717,7 +4711,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>3100000000000074</t>
+          <t>3174</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4774,7 +4768,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>3100000000000075</t>
+          <t>3175</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4831,7 +4825,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>3100000000000076</t>
+          <t>3176</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4888,7 +4882,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>3100000000000077</t>
+          <t>3177</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4945,7 +4939,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>3100000000000078</t>
+          <t>3178</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -5002,7 +4996,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>3100000000000079</t>
+          <t>3179</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -5059,7 +5053,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>3100000000000080</t>
+          <t>3180</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -5116,7 +5110,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>3100000000000081</t>
+          <t>3181</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -5173,7 +5167,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>3100000000000082</t>
+          <t>3182</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -5230,7 +5224,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>3100000000000083</t>
+          <t>3183</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -5287,7 +5281,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>3100000000000084</t>
+          <t>3184</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -5344,7 +5338,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>3100000000000085</t>
+          <t>3185</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -5401,7 +5395,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>3100000000000086</t>
+          <t>3186</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -5458,7 +5452,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>3100000000000087</t>
+          <t>3187</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -5515,7 +5509,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>3100000000000088</t>
+          <t>3188</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -5572,7 +5566,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>3100000000000089</t>
+          <t>3189</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -5629,7 +5623,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>3100000000000090</t>
+          <t>3190</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -5686,7 +5680,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>3100000000000091</t>
+          <t>3191</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -5743,7 +5737,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>3100000000000092</t>
+          <t>3192</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -5800,7 +5794,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>3100000000000093</t>
+          <t>3193</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5857,7 +5851,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>3100000000000094</t>
+          <t>3194</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5914,7 +5908,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>3100000000000095</t>
+          <t>3195</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5971,7 +5965,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>3100000000000096</t>
+          <t>3196</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -6028,7 +6022,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>3100000000000097</t>
+          <t>3197</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -6085,7 +6079,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>3100000000000098</t>
+          <t>3198</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -6142,7 +6136,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>3100000000000099</t>
+          <t>3199</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -6199,7 +6193,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>3100000000000100</t>
+          <t>31100</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -6256,7 +6250,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>3100000000000101</t>
+          <t>31101</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -6313,7 +6307,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>3100000000000102</t>
+          <t>31102</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -6370,7 +6364,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>3100000000000103</t>
+          <t>31103</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -6427,7 +6421,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>3100000000000104</t>
+          <t>31104</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -6484,7 +6478,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>3100000000000105</t>
+          <t>31105</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -6541,7 +6535,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>3100000000000106</t>
+          <t>31106</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -6598,7 +6592,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>3100000000000107</t>
+          <t>31107</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -6655,7 +6649,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>3100000000000108</t>
+          <t>31108</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -6712,7 +6706,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>3100000000000109</t>
+          <t>31109</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -6769,7 +6763,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>3100000000000110</t>
+          <t>31110</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -6826,7 +6820,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>3100000000000111</t>
+          <t>31111</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -6883,7 +6877,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>3100000000000112</t>
+          <t>31112</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -6940,7 +6934,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>3100000000000113</t>
+          <t>31113</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -6997,7 +6991,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>3100000000000114</t>
+          <t>31114</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -7054,7 +7048,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>3100000000000115</t>
+          <t>31115</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -7111,7 +7105,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>3100000000000116</t>
+          <t>31116</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -7168,7 +7162,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>3100000000000117</t>
+          <t>31117</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -7225,7 +7219,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>3100000000000118</t>
+          <t>31118</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -7282,7 +7276,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>3100000000000119</t>
+          <t>31119</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -7339,7 +7333,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>3100000000000120</t>
+          <t>31120</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -7396,7 +7390,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>3100000000000121</t>
+          <t>31121</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -7453,7 +7447,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>3100000000000122</t>
+          <t>31122</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -7510,7 +7504,7 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>3100000000000123</t>
+          <t>31123</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -7567,7 +7561,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>3100000000000124</t>
+          <t>31124</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -7624,7 +7618,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>3100000000000125</t>
+          <t>31125</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -7681,7 +7675,7 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>3100000000000126</t>
+          <t>31126</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -7738,7 +7732,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>3100000000000127</t>
+          <t>31127</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -7795,7 +7789,7 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>3100000000000128</t>
+          <t>31128</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -7852,7 +7846,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>3100000000000129</t>
+          <t>31129</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -7909,7 +7903,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>3100000000000130</t>
+          <t>31130</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -7966,7 +7960,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>3100000000000131</t>
+          <t>31131</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -8023,7 +8017,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>3100000000000132</t>
+          <t>31132</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -8080,7 +8074,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>3100000000000133</t>
+          <t>31133</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -8137,7 +8131,7 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>3100000000000134</t>
+          <t>31134</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -8194,7 +8188,7 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>3100000000000135</t>
+          <t>31135</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -8251,7 +8245,7 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>3100000000000136</t>
+          <t>31136</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -8308,7 +8302,7 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>3100000000000137</t>
+          <t>31137</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -8365,7 +8359,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>3100000000000138</t>
+          <t>31138</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -8422,7 +8416,7 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>3100000000000139</t>
+          <t>31139</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -8479,7 +8473,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>3100000000000140</t>
+          <t>31140</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -8536,7 +8530,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>3100000000000141</t>
+          <t>31141</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -8593,7 +8587,7 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>3100000000000142</t>
+          <t>31142</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -8650,7 +8644,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>3100000000000143</t>
+          <t>31143</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -8707,7 +8701,7 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>3100000000000144</t>
+          <t>31144</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -8764,7 +8758,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>3100000000000145</t>
+          <t>31145</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -8821,7 +8815,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>3100000000000146</t>
+          <t>31146</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -8878,7 +8872,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>3100000000000147</t>
+          <t>31147</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -8935,7 +8929,7 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>3100000000000148</t>
+          <t>31148</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -8992,7 +8986,7 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>3100000000000149</t>
+          <t>31149</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -9049,7 +9043,7 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>3100000000000150</t>
+          <t>31150</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -9106,7 +9100,7 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>3100000000000151</t>
+          <t>31151</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -9163,7 +9157,7 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>3100000000000152</t>
+          <t>31152</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -9220,7 +9214,7 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>3100000000000153</t>
+          <t>31153</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -9277,7 +9271,7 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>3100000000000154</t>
+          <t>31154</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -9334,7 +9328,7 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>3100000000000155</t>
+          <t>31155</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -9391,7 +9385,7 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>3100000000000156</t>
+          <t>31156</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -9448,7 +9442,7 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>3100000000000157</t>
+          <t>31157</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -9505,7 +9499,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>3100000000000158</t>
+          <t>31158</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -9562,7 +9556,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>3100000000000159</t>
+          <t>31159</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -9619,7 +9613,7 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>3100000000000160</t>
+          <t>31160</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -9676,7 +9670,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>3100000000000161</t>
+          <t>31161</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -9733,7 +9727,7 @@
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>3100000000000162</t>
+          <t>31162</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -9790,7 +9784,7 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>3100000000000163</t>
+          <t>31163</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -9847,7 +9841,7 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>3100000000000164</t>
+          <t>31164</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -9904,7 +9898,7 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>3100000000000165</t>
+          <t>31165</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -9961,7 +9955,7 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>3100000000000166</t>
+          <t>31166</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -10018,7 +10012,7 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>3100000000000167</t>
+          <t>31167</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -10075,7 +10069,7 @@
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>3100000000000168</t>
+          <t>31168</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -10132,7 +10126,7 @@
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>3100000000000169</t>
+          <t>31169</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -10189,7 +10183,7 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>3100000000000170</t>
+          <t>31170</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -10246,7 +10240,7 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>3100000000000171</t>
+          <t>31171</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -10303,7 +10297,7 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>3100000000000172</t>
+          <t>31172</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -10360,7 +10354,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>3100000000000173</t>
+          <t>31173</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -10417,7 +10411,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>3100000000000174</t>
+          <t>31174</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -10474,7 +10468,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>3100000000000175</t>
+          <t>31175</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -10531,7 +10525,7 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>3100000000000176</t>
+          <t>31176</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -10588,7 +10582,7 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>3100000000000177</t>
+          <t>31177</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -10645,7 +10639,7 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>3100000000000178</t>
+          <t>31178</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -10702,7 +10696,7 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>3100000000000179</t>
+          <t>31179</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -10759,7 +10753,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>3100000000000180</t>
+          <t>31180</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -10816,7 +10810,7 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>3100000000000181</t>
+          <t>31181</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -10873,7 +10867,7 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>3100000000000182</t>
+          <t>31182</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -10930,7 +10924,7 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>3100000000000183</t>
+          <t>31183</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -10987,7 +10981,7 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>3100000000000184</t>
+          <t>31184</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -11044,7 +11038,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>3100000000000185</t>
+          <t>31185</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -11101,7 +11095,7 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>3100000000000186</t>
+          <t>31186</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -11158,7 +11152,7 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>3100000000000187</t>
+          <t>31187</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -11215,7 +11209,7 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>3100000000000188</t>
+          <t>31188</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -11272,7 +11266,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>3100000000000189</t>
+          <t>31189</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -11329,7 +11323,7 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>3100000000000190</t>
+          <t>31190</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -11386,7 +11380,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>3100000000000191</t>
+          <t>31191</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -11443,7 +11437,7 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>3100000000000192</t>
+          <t>31192</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -11500,7 +11494,7 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>3100000000000193</t>
+          <t>31193</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -11557,7 +11551,7 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>3100000000000194</t>
+          <t>31194</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -11614,7 +11608,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>3100000000000195</t>
+          <t>31195</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -11671,7 +11665,7 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>3100000000000196</t>
+          <t>31196</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -11728,7 +11722,7 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>3100000000000197</t>
+          <t>31197</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -11785,7 +11779,7 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>3100000000000198</t>
+          <t>31198</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -11842,7 +11836,7 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>3100000000000199</t>
+          <t>31199</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -11899,7 +11893,7 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>3100000000000200</t>
+          <t>31200</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">

</xml_diff>